<commit_message>
[5 28] update arkusz_2.py
</commit_message>
<xml_diff>
--- a/day_5/dane_nowe.xlsx
+++ b/day_5/dane_nowe.xlsx
@@ -417,26 +417,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="B1" t="inlineStr">
         <is>
-          <t>Unnamed: 0</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
           <t>Sales Date</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Sales Person</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Amount</t>
         </is>
@@ -446,18 +441,15 @@
       <c r="A2" t="n">
         <v>0</v>
       </c>
-      <c r="B2" t="n">
-        <v>0</v>
-      </c>
-      <c r="C2" s="1" t="n">
+      <c r="B2" s="1" t="n">
         <v>43232</v>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>Sila Ahmed</t>
         </is>
       </c>
-      <c r="E2" t="n">
+      <c r="D2" t="n">
         <v>60000</v>
       </c>
     </row>

</xml_diff>